<commit_message>
Fix-Parameter der Speicherarten eingepflegt, Einlesen der Daten in Dataclasses in "Prognose_Speicher" definiert
</commit_message>
<xml_diff>
--- a/Quellen/ki_prompts_robin.xlsx
+++ b/Quellen/ki_prompts_robin.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Privat\HAW\Semester 3\IPJ 1\IPJ1-Pottkieker\Quellen\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A757458B-643A-4434-9138-2724408F0472}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5480F1E8-E791-4F10-9B09-DD2F0808C497}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
   <si>
     <t>df_ausbau = pd.concat([df_batterie, df_auto, df_schwungrad, df_wasserstoff, df_pump], axis=1)
 wie kann ich hier im resultierenden Dataframe die Spalten bezüglich des Datums nur einmal vorne haben und ansonsten nur die unterschiedlichen Speicherkapazitäten als weitere Spalten</t>
@@ -37,6 +37,9 @@
     speichername = f"Speicherkapazität {speicherart} [MWh]"
     df_2030[speichername] = speicher
 dieser code war auf 15 Minuten Intervalle ausgelegt, wie kann ich ihn jetzt so auslegen, dass die tägliche Wachstumsrate verwendet wird, aber trotzdem jeder eintrag im Dataframe, also alle 15 Minuten einen Wert zugeordnet bekommt?</t>
+  </si>
+  <si>
+    <t>ich kenne structures aus C, gibt es dafür ein äquivalent in python?</t>
   </si>
 </sst>
 </file>
@@ -360,7 +363,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A2"/>
+  <dimension ref="A1:A3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="107.7109375" style="1" customWidth="1"/>
@@ -376,6 +379,11 @@
         <v>1</v>
       </c>
     </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Dunkelflaute Implementation AUSGABE NOCH IN "Klassen"
</commit_message>
<xml_diff>
--- a/Quellen/ki_prompts_robin.xlsx
+++ b/Quellen/ki_prompts_robin.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Privat\HAW\Semester 3\IPJ 1\IPJ1-Pottkieker\Quellen\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48D97321-2B4B-4509-895F-5C8A7B757DBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8EAE83B-860F-4B06-9369-3F51D6674C3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t>df_ausbau = pd.concat([df_batterie, df_auto, df_schwungrad, df_wasserstoff, df_pump], axis=1)
 wie kann ich hier im resultierenden Dataframe die Spalten bezüglich des Datums nur einmal vorne haben und ansonsten nur die unterschiedlichen Speicherkapazitäten als weitere Spalten</t>
@@ -43,6 +43,12 @@
   </si>
   <si>
     <t>Wie kann ich dieses Dataframe jetzt am effizientesten sequentiell durchgehen?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">wie kann ich jetzt an genau den Tagen in der df_verlauf die den Tagen in der df_dunkelflaute entsprechen auf die Erzeugungswerte die Faktoren der Dunkelflaute anwenden? </t>
+  </si>
+  <si>
+    <t>wie kann ich diese sequentielle Schleife so anpassen, dass sie nur über einen bestimmten Bereich iteriert?</t>
   </si>
 </sst>
 </file>
@@ -366,7 +372,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A4"/>
+  <dimension ref="A1:A6"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="107.7109375" style="1" customWidth="1"/>
@@ -392,6 +398,16 @@
         <v>3</v>
       </c>
     </row>
+    <row r="5" spans="1:1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>